<commit_message>
Align roster template sample overalls with their listed ratings
The sample QB (overall 88) and RB (overall 84) rows had an overall
noticeably higher than the average of their own listed ratings (~79
and ~81 respectively) — not a functional bug since overall isn't
required to equal that average, but confusing as reference data since
it doesn't demonstrate the relationship a user would expect. Set both
to match, using the same rounding the importer's own overall fallback
uses, and regenerated the static public/templates/ files (the app
itself serves the template dynamically via /api/roster/template, so
this only affects those pre-generated files, not live downloads).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/roster-template.xlsx
+++ b/public/templates/roster-template.xlsx
@@ -932,7 +932,7 @@
         <v>71</v>
       </c>
       <c r="P2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="Q2">
         <v>62</v>
@@ -1027,7 +1027,7 @@
         <v>77</v>
       </c>
       <c r="P3">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="Q3">
         <v>88</v>

</xml_diff>